<commit_message>
Create template to compute Alpha for 4 coder
</commit_message>
<xml_diff>
--- a/P4 Pengembangan Kebutuhan Perangkat Lunak/A Elisitasi/A4 Coding/20261021 Lembar_Coding_Codebook_1_0_2 (Gemini 3.1 Pro).xlsx
+++ b/P4 Pengembangan Kebutuhan Perangkat Lunak/A Elisitasi/A4 Coding/20261021 Lembar_Coding_Codebook_1_0_2 (Gemini 3.1 Pro).xlsx
@@ -7566,7 +7566,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>226</v>
       </c>
@@ -7583,7 +7583,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
         <v>231</v>
       </c>
@@ -7597,7 +7597,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
         <v>231</v>
       </c>
@@ -7611,7 +7611,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
         <v>231</v>
       </c>
@@ -7625,7 +7625,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
         <v>231</v>
       </c>
@@ -7639,7 +7639,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>231</v>
       </c>
@@ -7653,7 +7653,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
         <v>231</v>
       </c>
@@ -7667,7 +7667,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>231</v>
       </c>
@@ -7681,7 +7681,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
         <v>231</v>
       </c>
@@ -7695,7 +7695,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
         <v>231</v>
       </c>
@@ -7709,7 +7709,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
         <v>231</v>
       </c>
@@ -7723,7 +7723,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
         <v>231</v>
       </c>
@@ -7737,7 +7737,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
         <v>231</v>
       </c>
@@ -7751,7 +7751,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
         <v>231</v>
       </c>
@@ -7765,7 +7765,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
         <v>231</v>
       </c>
@@ -7779,7 +7779,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
         <v>231</v>
       </c>
@@ -7793,7 +7793,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
         <v>231</v>
       </c>
@@ -7807,7 +7807,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
         <v>231</v>
       </c>
@@ -7821,7 +7821,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
         <v>231</v>
       </c>
@@ -7835,7 +7835,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
         <v>231</v>
       </c>
@@ -7852,7 +7852,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
         <v>231</v>
       </c>
@@ -7869,7 +7869,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
         <v>231</v>
       </c>
@@ -7886,7 +7886,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
         <v>231</v>
       </c>
@@ -7903,7 +7903,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
         <v>231</v>
       </c>
@@ -7920,7 +7920,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
         <v>231</v>
       </c>
@@ -7937,7 +7937,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
         <v>231</v>
       </c>
@@ -7954,7 +7954,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
         <v>231</v>
       </c>
@@ -7971,7 +7971,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
         <v>231</v>
       </c>
@@ -7988,7 +7988,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
         <v>231</v>
       </c>
@@ -8005,7 +8005,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
         <v>231</v>
       </c>
@@ -8022,7 +8022,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
         <v>231</v>
       </c>
@@ -8039,7 +8039,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
         <v>231</v>
       </c>
@@ -8056,7 +8056,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
         <v>231</v>
       </c>
@@ -8073,7 +8073,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
         <v>231</v>
       </c>
@@ -8090,7 +8090,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
         <v>231</v>
       </c>
@@ -8107,7 +8107,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
         <v>231</v>
       </c>
@@ -8124,7 +8124,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
         <v>231</v>
       </c>
@@ -8141,7 +8141,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
         <v>231</v>
       </c>
@@ -8158,7 +8158,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
         <v>231</v>
       </c>
@@ -8175,7 +8175,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
         <v>231</v>
       </c>
@@ -8192,7 +8192,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
         <v>231</v>
       </c>
@@ -8209,7 +8209,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
         <v>231</v>
       </c>
@@ -8226,7 +8226,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
         <v>231</v>
       </c>
@@ -8243,7 +8243,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
         <v>231</v>
       </c>
@@ -8260,7 +8260,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
         <v>231</v>
       </c>
@@ -8277,7 +8277,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
         <v>231</v>
       </c>
@@ -8294,7 +8294,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
         <v>231</v>
       </c>
@@ -8311,7 +8311,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="s">
         <v>231</v>
       </c>
@@ -8328,7 +8328,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
         <v>231</v>
       </c>
@@ -8345,7 +8345,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
         <v>231</v>
       </c>
@@ -8362,7 +8362,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
         <v>231</v>
       </c>
@@ -8379,7 +8379,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
         <v>231</v>
       </c>
@@ -8396,7 +8396,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="s">
         <v>231</v>
       </c>
@@ -8413,7 +8413,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
         <v>231</v>
       </c>
@@ -8430,7 +8430,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
         <v>231</v>
       </c>
@@ -8464,7 +8464,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
         <v>231</v>
       </c>
@@ -8478,7 +8478,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
         <v>231</v>
       </c>
@@ -8492,7 +8492,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="s">
         <v>360</v>
       </c>
@@ -8506,7 +8506,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
         <v>360</v>
       </c>

</xml_diff>